<commit_message>
feat: added a column that measures if the model correctly visually depicts board state
</commit_message>
<xml_diff>
--- a/hanoi_moves_programmatically_verified.xlsx
+++ b/hanoi_moves_programmatically_verified.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M256"/>
+  <dimension ref="A1:N256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,11 @@
           <t>Programmatic Match Human</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Visual State Match</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -537,6 +542,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -592,6 +602,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -643,6 +658,11 @@
         </is>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
@@ -702,6 +722,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -757,6 +782,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -812,6 +842,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -871,6 +906,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -926,6 +966,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -981,6 +1026,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1036,6 +1086,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1091,6 +1146,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1146,6 +1206,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1201,6 +1266,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1256,6 +1326,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1315,6 +1390,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1370,6 +1450,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1425,6 +1510,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1480,6 +1570,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1535,6 +1630,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1590,6 +1690,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1645,6 +1750,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1700,6 +1810,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1755,6 +1870,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1810,6 +1930,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1865,6 +1990,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1920,6 +2050,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1975,6 +2110,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2030,6 +2170,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2085,6 +2230,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2140,6 +2290,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2199,6 +2354,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2254,6 +2414,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2309,6 +2474,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2364,6 +2534,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2419,6 +2594,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2474,6 +2654,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2529,6 +2714,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2584,6 +2774,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2639,6 +2834,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2694,6 +2894,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2749,6 +2954,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2804,6 +3014,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2859,6 +3074,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2914,6 +3134,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2969,6 +3194,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3024,6 +3254,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3079,6 +3314,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3134,6 +3374,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3189,6 +3434,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3244,6 +3494,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3299,6 +3554,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3354,6 +3614,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3409,6 +3674,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3464,6 +3734,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3519,6 +3794,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3574,6 +3854,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3629,6 +3914,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3684,6 +3974,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3739,6 +4034,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3794,6 +4094,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3849,6 +4154,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3904,6 +4214,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3963,6 +4278,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4018,6 +4338,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4073,6 +4398,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4128,6 +4458,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4183,6 +4518,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4238,6 +4578,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4293,6 +4638,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4348,6 +4698,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4403,6 +4758,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4458,6 +4818,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4513,6 +4878,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4568,6 +4938,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4623,6 +4998,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4678,6 +5058,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4733,6 +5118,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4788,6 +5178,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -4843,6 +5238,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -4898,6 +5298,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -4953,6 +5358,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5008,6 +5418,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5063,6 +5478,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5118,6 +5538,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5173,6 +5598,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -5228,6 +5658,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -5283,6 +5718,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -5338,6 +5778,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5393,6 +5838,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -5448,6 +5898,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -5503,6 +5958,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -5558,6 +6018,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -5613,6 +6078,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -5668,6 +6138,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -5723,6 +6198,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -5778,6 +6258,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -5833,6 +6318,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -5888,6 +6378,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5943,6 +6438,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5998,6 +6498,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -6053,6 +6558,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -6108,6 +6618,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -6163,6 +6678,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -6218,6 +6738,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -6273,6 +6798,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -6328,6 +6858,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -6383,6 +6918,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -6438,6 +6978,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -6493,6 +7038,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -6548,6 +7098,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -6603,6 +7158,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -6658,6 +7218,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -6713,6 +7278,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -6768,6 +7338,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -6823,6 +7398,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -6878,6 +7458,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -6933,6 +7518,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -6988,6 +7578,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -7043,6 +7638,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -7098,6 +7698,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -7153,6 +7758,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -7208,6 +7818,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -7263,6 +7878,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -7318,6 +7938,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -7373,6 +7998,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -7428,6 +8058,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -7487,6 +8122,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -7542,6 +8182,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -7597,6 +8242,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -7652,6 +8302,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -7707,6 +8362,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -7762,6 +8422,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -7817,6 +8482,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -7872,6 +8542,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -7927,6 +8602,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -7982,6 +8662,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -8037,6 +8722,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -8092,6 +8782,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -8147,6 +8842,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -8202,6 +8902,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -8257,6 +8962,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -8312,6 +9022,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -8367,6 +9082,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -8422,6 +9142,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -8477,6 +9202,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -8532,6 +9262,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -8587,6 +9322,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -8642,6 +9382,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -8697,6 +9442,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -8752,6 +9502,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -8807,6 +9562,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -8862,6 +9622,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -8917,6 +9682,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -8972,6 +9742,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -9027,6 +9802,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -9082,6 +9862,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -9137,6 +9922,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -9192,6 +9982,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -9247,6 +10042,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -9302,6 +10102,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -9357,6 +10162,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -9412,6 +10222,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -9467,6 +10282,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -9522,6 +10342,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -9577,6 +10402,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -9632,6 +10462,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -9687,6 +10522,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -9742,6 +10582,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -9797,6 +10642,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -9852,6 +10702,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -9907,6 +10762,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -9962,6 +10822,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -10017,6 +10882,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -10072,6 +10942,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -10127,6 +11002,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -10182,6 +11062,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -10237,6 +11122,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -10292,6 +11182,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -10347,6 +11242,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -10402,6 +11302,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -10457,6 +11362,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -10512,6 +11422,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -10567,6 +11482,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -10622,6 +11542,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -10677,6 +11602,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -10732,6 +11662,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -10787,6 +11722,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -10842,6 +11782,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -10897,6 +11842,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -10952,6 +11902,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -11011,6 +11966,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -11066,6 +12026,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -11121,6 +12086,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -11176,6 +12146,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -11231,6 +12206,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -11286,6 +12266,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -11341,6 +12326,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -11396,6 +12386,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -11451,6 +12446,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -11506,6 +12506,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -11561,6 +12566,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -11616,6 +12626,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -11671,6 +12686,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -11726,6 +12746,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -11781,6 +12806,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -11836,6 +12866,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -11891,6 +12926,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -11946,6 +12986,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -12001,6 +13046,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -12056,6 +13106,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -12111,6 +13166,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -12166,6 +13226,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -12221,6 +13286,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -12276,6 +13346,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -12331,6 +13406,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -12386,6 +13466,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -12441,6 +13526,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -12496,6 +13586,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -12551,6 +13646,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -12606,6 +13706,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -12661,6 +13766,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -12716,6 +13826,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -12775,6 +13890,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -12830,6 +13950,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -12885,6 +14010,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -12940,6 +14070,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -12995,6 +14130,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -13050,6 +14190,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -13105,6 +14250,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -13160,6 +14310,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -13215,6 +14370,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -13270,6 +14430,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -13325,6 +14490,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -13380,6 +14550,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -13435,6 +14610,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -13490,6 +14670,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -13545,6 +14730,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -13600,6 +14790,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -13659,6 +14854,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -13714,6 +14914,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -13769,6 +14974,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -13824,6 +15034,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -13879,6 +15094,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -13934,6 +15154,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -13989,6 +15214,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -14044,6 +15274,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -14099,6 +15334,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -14154,6 +15394,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -14209,6 +15454,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -14264,6 +15514,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -14319,6 +15574,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -14374,6 +15634,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -14429,6 +15694,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -14484,6 +15754,11 @@
           <t>MATCH</t>
         </is>
       </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -14539,6 +15814,11 @@
         </is>
       </c>
       <c r="M256" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>

</xml_diff>